<commit_message>
Online Reporting Test Cases
</commit_message>
<xml_diff>
--- a/KatalonData/Bootstrap/VSP-Data.xlsx
+++ b/KatalonData/Bootstrap/VSP-Data.xlsx
@@ -1,30 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\Bootstrap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52FE45B-5B29-4174-8335-DBB320E07CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B6C668-5F6A-4826-96AB-3A1AED8B0564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2268" yWindow="1596" windowWidth="17280" windowHeight="9972" tabRatio="893" activeTab="3" xr2:uid="{F85E046C-D3FC-46F9-AA2F-5165245A7308}"/>
+    <workbookView xWindow="3168" yWindow="2268" windowWidth="17280" windowHeight="9972" tabRatio="893" firstSheet="10" activeTab="12" xr2:uid="{F85E046C-D3FC-46F9-AA2F-5165245A7308}"/>
   </bookViews>
   <sheets>
     <sheet name="CreateProfile" sheetId="1" r:id="rId1"/>
     <sheet name="VerifyViewProfile" sheetId="2" r:id="rId2"/>
     <sheet name="AddCCUI" sheetId="3" r:id="rId3"/>
     <sheet name="AddDeleteCCNotPrepopulated" sheetId="4" r:id="rId4"/>
-    <sheet name="AddDeleteCCPrepopulated" sheetId="5" r:id="rId5"/>
-    <sheet name="CreateModifyDeleteProfile" sheetId="6" r:id="rId6"/>
-    <sheet name="AddModifyDeleteCC" sheetId="7" r:id="rId7"/>
-    <sheet name="AddACHMRF" sheetId="8" r:id="rId8"/>
-    <sheet name="AddModifyDeleteACH" sheetId="9" r:id="rId9"/>
-    <sheet name="DC-CreateProfile" sheetId="10" r:id="rId10"/>
-    <sheet name="DC-CreateProfACH" sheetId="11" r:id="rId11"/>
-    <sheet name="SearchProfile" sheetId="12" r:id="rId12"/>
+    <sheet name="Sheet1" sheetId="13" r:id="rId5"/>
+    <sheet name="AddDeleteCCPrepopulated" sheetId="5" r:id="rId6"/>
+    <sheet name="CreateModifyDeleteProfile" sheetId="6" r:id="rId7"/>
+    <sheet name="AddModifyDeleteCC" sheetId="7" r:id="rId8"/>
+    <sheet name="AddACHMRF" sheetId="8" r:id="rId9"/>
+    <sheet name="AddModifyDeleteACH" sheetId="9" r:id="rId10"/>
+    <sheet name="DC-CreateProfile" sheetId="10" r:id="rId11"/>
+    <sheet name="DC-CreateProfACH" sheetId="11" r:id="rId12"/>
+    <sheet name="SearchProfile" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1283,7 +1284,7 @@
       <c r="T3" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X3" s="1" t="s">
@@ -1331,6 +1332,481 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{055BC8D0-1CFC-40D6-9313-A3584BAD2B30}">
+  <dimension ref="A1:AM4"/>
+  <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="13.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="29" width="14.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="32" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="25.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="16384" width="24.21875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="C2" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AK2" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AL2" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="AM2" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="T3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="W3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AB3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AL3" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="AM3" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="S4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="W4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AB4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC4" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AG4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AH4" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="AI4" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AJ4" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AK4" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="AL4" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="AM4" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F32B79-CCE8-401C-87BF-7A6DD5C015A7}">
   <dimension ref="A1:AL5"/>
   <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1525,7 +2001,7 @@
       <c r="S2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X2" s="1" t="s">
@@ -1617,7 +2093,7 @@
       <c r="S3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="W3" t="s">
+      <c r="W3" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X3" s="1" t="s">
@@ -1709,7 +2185,7 @@
       <c r="S4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="W4" t="s">
+      <c r="W4" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X4" s="1" t="s">
@@ -1801,7 +2277,7 @@
       <c r="S5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="W5" t="s">
+      <c r="W5" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X5" s="1" t="s">
@@ -1858,7 +2334,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1DBA674-D846-4D8B-BA8C-1C7D34927EB0}">
   <dimension ref="A1:AL4"/>
   <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2295,7 +2771,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A9BF8E7-6E86-4CC0-BBC0-582817F79C94}">
   <dimension ref="A1:J9"/>
   <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2522,7 +2998,7 @@
       <c r="H9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="1" t="s">
         <v>212</v>
       </c>
       <c r="J9" s="1" t="s">
@@ -3107,6 +3583,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D56AFAC1-9F33-4DC2-B99A-D4196214B827}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC310AF0-6FFB-4A8E-A2F9-ECD1411C076E}">
   <dimension ref="A1:AL2"/>
   <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3310,7 +3795,7 @@
       <c r="T2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X2" s="1" t="s">
@@ -3367,7 +3852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4940B053-892E-4D65-970C-387445E934F5}">
   <dimension ref="A1:AX2"/>
   <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3607,7 +4092,7 @@
       <c r="T2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X2" s="1" t="s">
@@ -3676,7 +4161,7 @@
       <c r="AS2" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AT2" s="1" t="s">
         <v>135</v>
       </c>
       <c r="AU2" s="1" t="s">
@@ -3700,7 +4185,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4C6E2C-C42D-471F-A066-CEBAB5BA432C}">
   <dimension ref="A1:AN2"/>
   <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3910,7 +4395,7 @@
       <c r="T2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="1" t="s">
         <v>54</v>
       </c>
       <c r="X2" s="1" t="s">
@@ -3973,7 +4458,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD29F020-32F0-46BA-9C78-0D5D38002911}">
   <dimension ref="A1:AH2"/>
   <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4145,479 +4630,4 @@
     <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{055BC8D0-1CFC-40D6-9313-A3584BAD2B30}">
-  <dimension ref="A1:AM4"/>
-  <sheetFormatPr defaultColWidth="24.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="11.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="4.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="26" width="13.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="29" width="14.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="32" width="12.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="25.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="16384" width="24.21875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:39" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="2" spans="1:39" x14ac:dyDescent="0.3">
-      <c r="C2" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="R2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="W2" t="s">
-        <v>54</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AD2" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG2" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="AI2" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="AJ2" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="AK2" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="AL2" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="AM2" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="3" spans="1:39" x14ac:dyDescent="0.3">
-      <c r="C3" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="P3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="R3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="S3" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="T3" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="W3" t="s">
-        <v>54</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AA3" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AB3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AC3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AD3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AF3" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG3" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="AI3" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="AJ3" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="AK3" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="AL3" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="AM3" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="4" spans="1:39" x14ac:dyDescent="0.3">
-      <c r="C4" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="S4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="W4" t="s">
-        <v>54</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AB4" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AC4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AD4" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AE4" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AF4" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AG4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AH4" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="AI4" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="AJ4" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="AK4" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="AL4" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="AM4" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter>
-    <oddFooter xml:space="preserve">&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Public </oddFooter>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>